<commit_message>
debug magnetic flux linkage
</commit_message>
<xml_diff>
--- a/FEMM_폴페어일렉트로닉스_dq_torque비교.xlsx
+++ b/FEMM_폴페어일렉트로닉스_dq_torque비교.xlsx
@@ -1385,11 +1385,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="-195327808"/>
-        <c:axId val="-195340864"/>
+        <c:axId val="1365717248"/>
+        <c:axId val="1365721056"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-195327808"/>
+        <c:axId val="1365717248"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1432,7 +1432,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-195340864"/>
+        <c:crossAx val="1365721056"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1440,7 +1440,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-195340864"/>
+        <c:axId val="1365721056"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1491,7 +1491,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-195327808"/>
+        <c:crossAx val="1365717248"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2273,11 +2273,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="-195332160"/>
-        <c:axId val="-195343040"/>
+        <c:axId val="1365719424"/>
+        <c:axId val="1365719968"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-195332160"/>
+        <c:axId val="1365719424"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2320,7 +2320,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-195343040"/>
+        <c:crossAx val="1365719968"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2328,7 +2328,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-195343040"/>
+        <c:axId val="1365719968"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2379,7 +2379,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-195332160"/>
+        <c:crossAx val="1365719424"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2982,34 +2982,34 @@
                   <c:v>-0.01</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>53.13</c:v>
+                  <c:v>44.53</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>105.68</c:v>
+                  <c:v>88.52</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>156.88</c:v>
+                  <c:v>127.42</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>202.83</c:v>
+                  <c:v>156.63999999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>245.33</c:v>
+                  <c:v>178.99</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>287.83999999999997</c:v>
+                  <c:v>197</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>325.43</c:v>
+                  <c:v>211.64</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>344.25</c:v>
+                  <c:v>224.47</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>363.08</c:v>
+                  <c:v>236</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>381.9</c:v>
+                  <c:v>246.71</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3094,34 +3094,34 @@
                   <c:v>-0.01</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.62</c:v>
+                  <c:v>-4.28</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.25</c:v>
+                  <c:v>-8.6300000000000008</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>13.6</c:v>
+                  <c:v>-12.92</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>17.829999999999998</c:v>
+                  <c:v>-16.489999999999998</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>22.29</c:v>
+                  <c:v>-18.63</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>24.24</c:v>
+                  <c:v>-18.71</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>25.91</c:v>
+                  <c:v>-18.309999999999999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>29.62</c:v>
+                  <c:v>-17.940000000000001</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>33.32</c:v>
+                  <c:v>-17.88</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>37.03</c:v>
+                  <c:v>-18.16</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3137,11 +3137,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="-195342496"/>
-        <c:axId val="-195340320"/>
+        <c:axId val="1365723776"/>
+        <c:axId val="1365722144"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-195342496"/>
+        <c:axId val="1365723776"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3184,7 +3184,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-195340320"/>
+        <c:crossAx val="1365722144"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3192,7 +3192,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-195340320"/>
+        <c:axId val="1365722144"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3243,7 +3243,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-195342496"/>
+        <c:crossAx val="1365723776"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3763,61 +3763,61 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
                 <c:pt idx="0">
-                  <c:v>381.9</c:v>
+                  <c:v>246.71</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>381.19</c:v>
+                  <c:v>245.62</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>379.04</c:v>
+                  <c:v>243.65</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>375.49</c:v>
+                  <c:v>240.75</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>370.55</c:v>
+                  <c:v>236.77</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>362.26</c:v>
+                  <c:v>231.46</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>344.61</c:v>
+                  <c:v>224.31</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>325.20999999999998</c:v>
+                  <c:v>214.75</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>304.19</c:v>
+                  <c:v>201.61</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>279.95</c:v>
+                  <c:v>183.39</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>251.92</c:v>
+                  <c:v>160.44999999999999</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>222.06</c:v>
+                  <c:v>134.5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>190.94</c:v>
+                  <c:v>105.93</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>159.11000000000001</c:v>
+                  <c:v>76.459999999999994</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>127.1</c:v>
+                  <c:v>50.37</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>95.52</c:v>
+                  <c:v>27.47</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>66.34</c:v>
+                  <c:v>4.9400000000000004</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>37.03</c:v>
+                  <c:v>-18.16</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-0.02</c:v>
+                  <c:v>-44.19</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4243,61 +4243,61 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
                 <c:pt idx="0">
-                  <c:v>53.13</c:v>
+                  <c:v>44.53</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>52.92</c:v>
+                  <c:v>43.62</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>52.32</c:v>
+                  <c:v>42.37</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>51.32</c:v>
+                  <c:v>40.81</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>49.92</c:v>
+                  <c:v>38.93</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>48.15</c:v>
+                  <c:v>36.75</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>46.01</c:v>
+                  <c:v>34.29</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>43.52</c:v>
+                  <c:v>31.58</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>40.700000000000003</c:v>
+                  <c:v>28.63</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>37.56</c:v>
+                  <c:v>25.48</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>34.15</c:v>
+                  <c:v>22.14</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>30.47</c:v>
+                  <c:v>18.64</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>26.56</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>22.45</c:v>
+                  <c:v>11.25</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>18.16</c:v>
+                  <c:v>7.42</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>13.74</c:v>
+                  <c:v>3.54</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>9.2200000000000006</c:v>
+                  <c:v>-0.37</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>4.62</c:v>
+                  <c:v>-4.28</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-0.01</c:v>
+                  <c:v>-8.15</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4313,11 +4313,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="-195335968"/>
-        <c:axId val="-195332704"/>
+        <c:axId val="1365724320"/>
+        <c:axId val="1365723232"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-195335968"/>
+        <c:axId val="1365724320"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4360,7 +4360,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-195332704"/>
+        <c:crossAx val="1365723232"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4368,7 +4368,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-195332704"/>
+        <c:axId val="1365723232"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4419,7 +4419,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-195335968"/>
+        <c:crossAx val="1365724320"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4924,11 +4924,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="-195341952"/>
-        <c:axId val="-195339232"/>
+        <c:axId val="1365724864"/>
+        <c:axId val="1365725952"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-195341952"/>
+        <c:axId val="1365724864"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4970,7 +4970,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-195339232"/>
+        <c:crossAx val="1365725952"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4978,7 +4978,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-195339232"/>
+        <c:axId val="1365725952"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5029,7 +5029,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-195341952"/>
+        <c:crossAx val="1365724864"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5387,11 +5387,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="-195329984"/>
-        <c:axId val="-195335424"/>
+        <c:axId val="1141607216"/>
+        <c:axId val="1141600688"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-195329984"/>
+        <c:axId val="1141607216"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5433,7 +5433,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-195335424"/>
+        <c:crossAx val="1141600688"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5441,7 +5441,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-195335424"/>
+        <c:axId val="1141600688"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5492,7 +5492,7 @@
             <a:endParaRPr lang="ko-KR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-195329984"/>
+        <c:crossAx val="1141607216"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -11707,34 +11707,34 @@
         <v>-0.01</v>
       </c>
       <c r="P2">
-        <v>53.13</v>
+        <v>44.53</v>
       </c>
       <c r="Q2">
-        <v>105.68</v>
+        <v>88.52</v>
       </c>
       <c r="R2">
-        <v>156.88</v>
+        <v>127.42</v>
       </c>
       <c r="S2">
-        <v>202.83</v>
+        <v>156.63999999999999</v>
       </c>
       <c r="T2">
-        <v>245.33</v>
+        <v>178.99</v>
       </c>
       <c r="U2">
-        <v>287.83999999999997</v>
+        <v>197</v>
       </c>
       <c r="V2">
-        <v>325.43</v>
+        <v>211.64</v>
       </c>
       <c r="W2">
-        <v>344.25</v>
+        <v>224.47</v>
       </c>
       <c r="X2">
-        <v>363.08</v>
+        <v>236</v>
       </c>
       <c r="Y2">
-        <v>381.9</v>
+        <v>246.71</v>
       </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.3">
@@ -11781,34 +11781,34 @@
         <v>-0.01</v>
       </c>
       <c r="P3">
-        <v>52.92</v>
+        <v>43.62</v>
       </c>
       <c r="Q3">
-        <v>105.29</v>
+        <v>86.7</v>
       </c>
       <c r="R3">
-        <v>156.30000000000001</v>
+        <v>124.97</v>
       </c>
       <c r="S3">
-        <v>202.18</v>
+        <v>154.63</v>
       </c>
       <c r="T3">
-        <v>244.53</v>
+        <v>177.33</v>
       </c>
       <c r="U3">
-        <v>286.87</v>
+        <v>195.56</v>
       </c>
       <c r="V3">
-        <v>322.89999999999998</v>
+        <v>210.33</v>
       </c>
       <c r="W3">
-        <v>343.68</v>
+        <v>223.27</v>
       </c>
       <c r="X3">
-        <v>362.43</v>
+        <v>234.88</v>
       </c>
       <c r="Y3">
-        <v>381.19</v>
+        <v>245.62</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.3">
@@ -11855,34 +11855,34 @@
         <v>-0.01</v>
       </c>
       <c r="P4">
-        <v>52.32</v>
+        <v>42.37</v>
       </c>
       <c r="Q4">
-        <v>104.13</v>
+        <v>84.22</v>
       </c>
       <c r="R4">
-        <v>154.55000000000001</v>
+        <v>121.56</v>
       </c>
       <c r="S4">
-        <v>200.25</v>
+        <v>151.47999999999999</v>
       </c>
       <c r="T4">
-        <v>242.11</v>
+        <v>174.63</v>
       </c>
       <c r="U4">
-        <v>283.95999999999998</v>
+        <v>193.19</v>
       </c>
       <c r="V4">
-        <v>316.31</v>
+        <v>208.12</v>
       </c>
       <c r="W4">
-        <v>341.96</v>
+        <v>221.19</v>
       </c>
       <c r="X4">
-        <v>360.5</v>
+        <v>232.89</v>
       </c>
       <c r="Y4">
-        <v>379.04</v>
+        <v>243.65</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.3">
@@ -11929,34 +11929,34 @@
         <v>-0.01</v>
       </c>
       <c r="P5">
-        <v>51.32</v>
+        <v>40.81</v>
       </c>
       <c r="Q5">
-        <v>102.13</v>
+        <v>81.12</v>
       </c>
       <c r="R5">
-        <v>151.65</v>
+        <v>117.21</v>
       </c>
       <c r="S5">
-        <v>196.47</v>
+        <v>146.97</v>
       </c>
       <c r="T5">
-        <v>238.09</v>
+        <v>170.74</v>
       </c>
       <c r="U5">
-        <v>279.14999999999998</v>
+        <v>189.72</v>
       </c>
       <c r="V5">
-        <v>308.18</v>
+        <v>204.9</v>
       </c>
       <c r="W5">
-        <v>336.04</v>
+        <v>218.11</v>
       </c>
       <c r="X5">
-        <v>357.3</v>
+        <v>229.95</v>
       </c>
       <c r="Y5">
-        <v>375.49</v>
+        <v>240.75</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.3">
@@ -12003,34 +12003,34 @@
         <v>-0.01</v>
       </c>
       <c r="P6">
-        <v>49.92</v>
+        <v>38.93</v>
       </c>
       <c r="Q6">
-        <v>99.3</v>
+        <v>77.41</v>
       </c>
       <c r="R6">
-        <v>147.55000000000001</v>
+        <v>111.94</v>
       </c>
       <c r="S6">
-        <v>190.72</v>
+        <v>141.02000000000001</v>
       </c>
       <c r="T6">
-        <v>232.51</v>
+        <v>165.37</v>
       </c>
       <c r="U6">
-        <v>272.08999999999997</v>
+        <v>184.91</v>
       </c>
       <c r="V6">
-        <v>298.57</v>
+        <v>200.46</v>
       </c>
       <c r="W6">
-        <v>325.05</v>
+        <v>213.83</v>
       </c>
       <c r="X6">
-        <v>351.53</v>
+        <v>225.86</v>
       </c>
       <c r="Y6">
-        <v>370.55</v>
+        <v>236.77</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.3">
@@ -12077,34 +12077,34 @@
         <v>-0.01</v>
       </c>
       <c r="P7">
-        <v>48.15</v>
+        <v>36.75</v>
       </c>
       <c r="Q7">
-        <v>95.73</v>
+        <v>73.13</v>
       </c>
       <c r="R7">
-        <v>142.25</v>
+        <v>105.83</v>
       </c>
       <c r="S7">
-        <v>183.65</v>
+        <v>133.72999999999999</v>
       </c>
       <c r="T7">
-        <v>225.05</v>
+        <v>158.1</v>
       </c>
       <c r="U7">
-        <v>262.64</v>
+        <v>178.4</v>
       </c>
       <c r="V7">
-        <v>287.55</v>
+        <v>194.54</v>
       </c>
       <c r="W7">
-        <v>312.45</v>
+        <v>208.12</v>
       </c>
       <c r="X7">
-        <v>337.35</v>
+        <v>220.32</v>
       </c>
       <c r="Y7">
-        <v>362.26</v>
+        <v>231.46</v>
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.3">
@@ -12151,34 +12151,34 @@
         <v>-0.01</v>
       </c>
       <c r="P8">
-        <v>46.01</v>
+        <v>34.29</v>
       </c>
       <c r="Q8">
-        <v>91.43</v>
+        <v>68.290000000000006</v>
       </c>
       <c r="R8">
-        <v>136</v>
+        <v>98.99</v>
       </c>
       <c r="S8">
-        <v>175.32</v>
+        <v>125.2</v>
       </c>
       <c r="T8">
-        <v>214.64</v>
+        <v>148.77000000000001</v>
       </c>
       <c r="U8">
-        <v>252.06</v>
+        <v>169.57</v>
       </c>
       <c r="V8">
-        <v>275.2</v>
+        <v>186.64</v>
       </c>
       <c r="W8">
-        <v>298.33999999999997</v>
+        <v>200.61</v>
       </c>
       <c r="X8">
-        <v>321.47000000000003</v>
+        <v>212.97</v>
       </c>
       <c r="Y8">
-        <v>344.61</v>
+        <v>224.31</v>
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.3">
@@ -12225,34 +12225,34 @@
         <v>-0.01</v>
       </c>
       <c r="P9">
-        <v>43.52</v>
+        <v>31.58</v>
       </c>
       <c r="Q9">
-        <v>86.46</v>
+        <v>62.93</v>
       </c>
       <c r="R9">
-        <v>128.63</v>
+        <v>91.44</v>
       </c>
       <c r="S9">
-        <v>165.8</v>
+        <v>115.61</v>
       </c>
       <c r="T9">
-        <v>202.74</v>
+        <v>137.68</v>
       </c>
       <c r="U9">
-        <v>238.38</v>
+        <v>157.94</v>
       </c>
       <c r="V9">
-        <v>261.61</v>
+        <v>175.76</v>
       </c>
       <c r="W9">
-        <v>282.81</v>
+        <v>190.49</v>
       </c>
       <c r="X9">
-        <v>304.01</v>
+        <v>203.23</v>
       </c>
       <c r="Y9">
-        <v>325.20999999999998</v>
+        <v>214.75</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.3">
@@ -12299,34 +12299,34 @@
         <v>-0.01</v>
       </c>
       <c r="P10">
-        <v>40.700000000000003</v>
+        <v>28.63</v>
       </c>
       <c r="Q10">
-        <v>80.84</v>
+        <v>57.09</v>
       </c>
       <c r="R10">
-        <v>120.38</v>
+        <v>83.23</v>
       </c>
       <c r="S10">
-        <v>155.04</v>
+        <v>105.17</v>
       </c>
       <c r="T10">
-        <v>189.43</v>
+        <v>125.17</v>
       </c>
       <c r="U10">
-        <v>223.34</v>
+        <v>143.94999999999999</v>
       </c>
       <c r="V10">
-        <v>244.16</v>
+        <v>161.36000000000001</v>
       </c>
       <c r="W10">
-        <v>264.97000000000003</v>
+        <v>176.55</v>
       </c>
       <c r="X10">
-        <v>285.08999999999997</v>
+        <v>189.69</v>
       </c>
       <c r="Y10">
-        <v>304.19</v>
+        <v>201.61</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.3">
@@ -12373,34 +12373,34 @@
         <v>-0.01</v>
       </c>
       <c r="P11">
-        <v>37.56</v>
+        <v>25.48</v>
       </c>
       <c r="Q11">
-        <v>74.62</v>
+        <v>50.8</v>
       </c>
       <c r="R11">
-        <v>111.11</v>
+        <v>74.36</v>
       </c>
       <c r="S11">
-        <v>142.97</v>
+        <v>93.96</v>
       </c>
       <c r="T11">
-        <v>174.62</v>
+        <v>111.61</v>
       </c>
       <c r="U11">
-        <v>206.17</v>
+        <v>128.24</v>
       </c>
       <c r="V11">
-        <v>225.5</v>
+        <v>144.04</v>
       </c>
       <c r="W11">
-        <v>243.65</v>
+        <v>158.72999999999999</v>
       </c>
       <c r="X11">
-        <v>261.8</v>
+        <v>171.67</v>
       </c>
       <c r="Y11">
-        <v>279.95</v>
+        <v>183.39</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.3">
@@ -12447,34 +12447,34 @@
         <v>-0.01</v>
       </c>
       <c r="P12">
-        <v>34.15</v>
+        <v>22.14</v>
       </c>
       <c r="Q12">
-        <v>67.84</v>
+        <v>44.12</v>
       </c>
       <c r="R12">
-        <v>100.94</v>
+        <v>64.86</v>
       </c>
       <c r="S12">
-        <v>129.94</v>
+        <v>82.06</v>
       </c>
       <c r="T12">
-        <v>158.33000000000001</v>
+        <v>97.17</v>
       </c>
       <c r="U12">
-        <v>186.72</v>
+        <v>111.34</v>
       </c>
       <c r="V12">
-        <v>205.6</v>
+        <v>124.88</v>
       </c>
       <c r="W12">
-        <v>221.14</v>
+        <v>137.81</v>
       </c>
       <c r="X12">
-        <v>236.58</v>
+        <v>149.80000000000001</v>
       </c>
       <c r="Y12">
-        <v>251.92</v>
+        <v>160.44999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.3">
@@ -12521,34 +12521,34 @@
         <v>-0.01</v>
       </c>
       <c r="P13">
-        <v>30.47</v>
+        <v>18.64</v>
       </c>
       <c r="Q13">
-        <v>60.56</v>
+        <v>37.090000000000003</v>
       </c>
       <c r="R13">
-        <v>90.02</v>
+        <v>54.74</v>
       </c>
       <c r="S13">
-        <v>116.05</v>
+        <v>69.5</v>
       </c>
       <c r="T13">
-        <v>140.97</v>
+        <v>81.97</v>
       </c>
       <c r="U13">
-        <v>165.88</v>
+        <v>93.48</v>
       </c>
       <c r="V13">
-        <v>184.48</v>
+        <v>104.43</v>
       </c>
       <c r="W13">
-        <v>197</v>
+        <v>114.98</v>
       </c>
       <c r="X13">
-        <v>209.53</v>
+        <v>125.09</v>
       </c>
       <c r="Y13">
-        <v>222.06</v>
+        <v>134.5</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.3">
@@ -12595,34 +12595,34 @@
         <v>-0.01</v>
       </c>
       <c r="P14">
-        <v>26.56</v>
+        <v>15</v>
       </c>
       <c r="Q14">
-        <v>52.83</v>
+        <v>29.77</v>
       </c>
       <c r="R14">
-        <v>78.430000000000007</v>
+        <v>44.09</v>
       </c>
       <c r="S14">
-        <v>101.4</v>
+        <v>56.31</v>
       </c>
       <c r="T14">
-        <v>122.65</v>
+        <v>66.09</v>
       </c>
       <c r="U14">
-        <v>143.9</v>
+        <v>74.83</v>
       </c>
       <c r="V14">
-        <v>162.69999999999999</v>
+        <v>83.01</v>
       </c>
       <c r="W14">
-        <v>172.11</v>
+        <v>90.87</v>
       </c>
       <c r="X14">
-        <v>181.53</v>
+        <v>98.52</v>
       </c>
       <c r="Y14">
-        <v>190.94</v>
+        <v>105.93</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.3">
@@ -12669,34 +12669,34 @@
         <v>-0.01</v>
       </c>
       <c r="P15">
-        <v>22.45</v>
+        <v>11.25</v>
       </c>
       <c r="Q15">
-        <v>44.71</v>
+        <v>22.25</v>
       </c>
       <c r="R15">
-        <v>66.25</v>
+        <v>32.979999999999997</v>
       </c>
       <c r="S15">
-        <v>86.11</v>
+        <v>42.44</v>
       </c>
       <c r="T15">
-        <v>103.53</v>
+        <v>49.58</v>
       </c>
       <c r="U15">
-        <v>120.96</v>
+        <v>55.59</v>
       </c>
       <c r="V15">
-        <v>138.38999999999999</v>
+        <v>61.1</v>
       </c>
       <c r="W15">
-        <v>146.65</v>
+        <v>66.34</v>
       </c>
       <c r="X15">
-        <v>152.88</v>
+        <v>71.44</v>
       </c>
       <c r="Y15">
-        <v>159.11000000000001</v>
+        <v>76.459999999999994</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.3">
@@ -12743,34 +12743,34 @@
         <v>-0.01</v>
       </c>
       <c r="P16">
-        <v>18.16</v>
+        <v>7.42</v>
       </c>
       <c r="Q16">
-        <v>36.270000000000003</v>
+        <v>14.59</v>
       </c>
       <c r="R16">
-        <v>53.58</v>
+        <v>21.54</v>
       </c>
       <c r="S16">
-        <v>70.28</v>
+        <v>27.88</v>
       </c>
       <c r="T16">
-        <v>83.75</v>
+        <v>32.72</v>
       </c>
       <c r="U16">
-        <v>97.22</v>
+        <v>36.32</v>
       </c>
       <c r="V16">
-        <v>110.69</v>
+        <v>39.479999999999997</v>
       </c>
       <c r="W16">
-        <v>120.8</v>
+        <v>42.63</v>
       </c>
       <c r="X16">
-        <v>123.9</v>
+        <v>46.25</v>
       </c>
       <c r="Y16">
-        <v>127.1</v>
+        <v>50.37</v>
       </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.3">
@@ -12817,34 +12817,34 @@
         <v>-0.01</v>
       </c>
       <c r="P17">
-        <v>13.74</v>
+        <v>3.54</v>
       </c>
       <c r="Q17">
-        <v>27.49</v>
+        <v>6.86</v>
       </c>
       <c r="R17">
-        <v>40.520000000000003</v>
+        <v>9.99</v>
       </c>
       <c r="S17">
-        <v>53.47</v>
+        <v>12.98</v>
       </c>
       <c r="T17">
-        <v>63.45</v>
+        <v>15.58</v>
       </c>
       <c r="U17">
-        <v>72.95</v>
+        <v>17.28</v>
       </c>
       <c r="V17">
-        <v>82.66</v>
+        <v>19.22</v>
       </c>
       <c r="W17">
-        <v>92.36</v>
+        <v>21.85</v>
       </c>
       <c r="X17">
-        <v>95.48</v>
+        <v>24.64</v>
       </c>
       <c r="Y17">
-        <v>95.52</v>
+        <v>27.47</v>
       </c>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.3">
@@ -12891,34 +12891,34 @@
         <v>-0.01</v>
       </c>
       <c r="P18">
-        <v>9.2200000000000006</v>
+        <v>-0.37</v>
       </c>
       <c r="Q18">
-        <v>18.440000000000001</v>
+        <v>-0.9</v>
       </c>
       <c r="R18">
-        <v>27.15</v>
+        <v>-1.55</v>
       </c>
       <c r="S18">
-        <v>35.659999999999997</v>
+        <v>-1.87</v>
       </c>
       <c r="T18">
-        <v>43.06</v>
+        <v>-1.8</v>
       </c>
       <c r="U18">
-        <v>48.73</v>
+        <v>-0.79</v>
       </c>
       <c r="V18">
-        <v>54.39</v>
+        <v>0.78</v>
       </c>
       <c r="W18">
-        <v>60.06</v>
+        <v>2.2400000000000002</v>
       </c>
       <c r="X18">
-        <v>66.41</v>
+        <v>3.63</v>
       </c>
       <c r="Y18">
-        <v>66.34</v>
+        <v>4.9400000000000004</v>
       </c>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.3">
@@ -12965,34 +12965,34 @@
         <v>-0.01</v>
       </c>
       <c r="P19">
-        <v>4.62</v>
+        <v>-4.28</v>
       </c>
       <c r="Q19">
-        <v>9.25</v>
+        <v>-8.6300000000000008</v>
       </c>
       <c r="R19">
-        <v>13.6</v>
+        <v>-12.92</v>
       </c>
       <c r="S19">
-        <v>17.829999999999998</v>
+        <v>-16.489999999999998</v>
       </c>
       <c r="T19">
-        <v>22.29</v>
+        <v>-18.63</v>
       </c>
       <c r="U19">
-        <v>24.24</v>
+        <v>-18.71</v>
       </c>
       <c r="V19">
-        <v>25.91</v>
+        <v>-18.309999999999999</v>
       </c>
       <c r="W19">
-        <v>29.62</v>
+        <v>-17.940000000000001</v>
       </c>
       <c r="X19">
-        <v>33.32</v>
+        <v>-17.88</v>
       </c>
       <c r="Y19">
-        <v>37.03</v>
+        <v>-18.16</v>
       </c>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.3">
@@ -13039,34 +13039,34 @@
         <v>-0.01</v>
       </c>
       <c r="P20">
-        <v>-0.01</v>
+        <v>-8.15</v>
       </c>
       <c r="Q20">
-        <v>-0.01</v>
+        <v>-16.29</v>
       </c>
       <c r="R20">
-        <v>-0.02</v>
+        <v>-24.05</v>
       </c>
       <c r="S20">
-        <v>-0.02</v>
+        <v>-30.65</v>
       </c>
       <c r="T20">
-        <v>-0.02</v>
+        <v>-34.619999999999997</v>
       </c>
       <c r="U20">
-        <v>-0.02</v>
+        <v>-36.979999999999997</v>
       </c>
       <c r="V20">
-        <v>-0.02</v>
+        <v>-38.9</v>
       </c>
       <c r="W20">
-        <v>-0.02</v>
+        <v>-40.67</v>
       </c>
       <c r="X20">
-        <v>-0.02</v>
+        <v>-42.41</v>
       </c>
       <c r="Y20">
-        <v>-0.02</v>
+        <v>-44.19</v>
       </c>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.3">

</xml_diff>